<commit_message>
Add core-book manuscript (no PDFs); sync F1 v0.1.9 re-pin
</commit_message>
<xml_diff>
--- a/tables/achievements.xlsx
+++ b/tables/achievements.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Achievements" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Achievements'!$A$1:$J$1824</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Achievements'!$A$1:$J$1827</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1824"/>
+  <dimension ref="A1:J1827"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -94821,8 +94821,164 @@
         </is>
       </c>
     </row>
+    <row r="1825">
+      <c r="A1825" t="inlineStr">
+        <is>
+          <t>ACH-1824</t>
+        </is>
+      </c>
+      <c r="B1825" t="inlineStr">
+        <is>
+          <t>Not Unpacking</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr">
+        <is>
+          <t>Take a stairwell down within one in-game hour of arriving on a floor.</t>
+        </is>
+      </c>
+      <c r="D1825" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="E1825" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="F1825" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="G1825" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H1825" t="inlineStr">
+        <is>
+          <t>GM-tailored box + Title: Not Unpacking (floor caps apply; Silver ceiling on Floors 1-2)</t>
+        </is>
+      </c>
+      <c r="I1825" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J1825" t="inlineStr">
+        <is>
+          <t>Canon ref A-044 (CANON-LEDGER, VERIFIED). Not attainable on Floor 1: stairwells open about 32 h in (M-276) and early descent is stasis (M-277, decision 026). Snark: "Sixty minutes. The welcome mat is still warm. We will be telling the sponsors you were efficient."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" t="inlineStr">
+        <is>
+          <t>ACH-1825</t>
+        </is>
+      </c>
+      <c r="B1826" t="inlineStr">
+        <is>
+          <t>Down Is a Direction</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr">
+        <is>
+          <t>Find a stairwell down to the next floor (first time per Crawler).</t>
+        </is>
+      </c>
+      <c r="D1826" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="E1826" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="F1826" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G1826" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H1826" t="inlineStr">
+        <is>
+          <t>— (snark only)</t>
+        </is>
+      </c>
+      <c r="I1826" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J1826" t="inlineStr">
+        <is>
+          <t>Canon ref A-139 (CANON-LEDGER, VERIFIED; canon gives no prize). On Floor 1 the real stairwell is behind the Z10 stage (M-275); Z7 Big Green EXIT is bait. Snark: "Congratulations! You have located the floor's least decorative feature. It goes down. So do you, eventually."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" t="inlineStr">
+        <is>
+          <t>ACH-1826</t>
+        </is>
+      </c>
+      <c r="B1827" t="inlineStr">
+        <is>
+          <t>Left Before the Cake</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr">
+        <is>
+          <t>Go down a stairwell more than six in-game hours before the floor collapses.</t>
+        </is>
+      </c>
+      <c r="D1827" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="E1827" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="F1827" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G1827" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H1827" t="inlineStr">
+        <is>
+          <t>Title: Left Before the Cake (snark-only allowed; GM may add a small reward inside floor caps)</t>
+        </is>
+      </c>
+      <c r="I1827" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J1827" t="inlineStr">
+        <is>
+          <t>Canon ref A-151 (CANON-LEDGER, WIKI-ONLY). Early descent means stasis until the collapse (M-277); on Floor 1 attainable only in the stasis form (decision 026). Snark: "Leaving the party at nine-fifteen? Bold. Please enjoy the waiting room while everyone else has fun without you."</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1824"/>
+  <autoFilter ref="A1:J1827"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Include Core Book PDF build
</commit_message>
<xml_diff>
--- a/tables/achievements.xlsx
+++ b/tables/achievements.xlsx
@@ -446,28 +446,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Total achievements: 1823</t>
+          <t>Total achievements: 1826</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>With rewards: 1671</t>
+          <t>With rewards: 1673</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Brag-only (no reward): 152</t>
+          <t>Brag-only (no reward): 153</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Canon flavor tagged: 55</t>
+          <t>Canon flavor tagged: 58</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1039</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="9">
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="10">
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12">
@@ -94834,7 +94834,7 @@
       </c>
       <c r="C1825" t="inlineStr">
         <is>
-          <t>Take a stairwell down within one in-game hour of arriving on a floor.</t>
+          <t>Take a stairwell down within one in-game hour of arriving on a floor (once per Crawler, ever).</t>
         </is>
       </c>
       <c r="D1825" t="inlineStr">
@@ -94859,7 +94859,7 @@
       </c>
       <c r="H1825" t="inlineStr">
         <is>
-          <t>GM-tailored box + Title: Not Unpacking (floor caps apply; Silver ceiling on Floors 1-2)</t>
+          <t>Platinum box (canon-faithful to A-044; floor caps apply: if the floor's box ceiling is lower, the GM gives the ceiling tier and logs it) + Title: Not Unpacking. Never a Legendary box; never counts against the campaign Legendary box cap of 2 (core §4.5).</t>
         </is>
       </c>
       <c r="I1825" t="inlineStr">
@@ -94869,7 +94869,7 @@
       </c>
       <c r="J1825" t="inlineStr">
         <is>
-          <t>Canon ref A-044 (CANON-LEDGER, VERIFIED). Not attainable on Floor 1: stairwells open about 32 h in (M-276) and early descent is stasis (M-277, decision 026). Snark: "Sixty minutes. The welcome mat is still warm. We will be telling the sponsors you were efficient."</t>
+          <t>Canon ref A-044 (CANON-LEDGER, VERIFIED). Not attainable on Floor 1: stairwells open about 32 h in (M-276) and early descent is stasis (M-277, decision 026). Snark: "Sixty minutes. The welcome mat is still warm. We will be telling the sponsors you were efficient." Rarity tag Legendary is the achievement's rarity, not a box tier.</t>
         </is>
       </c>
     </row>
@@ -94886,7 +94886,7 @@
       </c>
       <c r="C1826" t="inlineStr">
         <is>
-          <t>Find a stairwell down to the next floor (first time per Crawler).</t>
+          <t>Find a stairwell down to the next floor (once per Crawler, ever).</t>
         </is>
       </c>
       <c r="D1826" t="inlineStr">
@@ -94938,7 +94938,7 @@
       </c>
       <c r="C1827" t="inlineStr">
         <is>
-          <t>Go down a stairwell more than six in-game hours before the floor collapses.</t>
+          <t>Go down a stairwell more than six in-game hours before the floor collapses (once per Crawler, ever).</t>
         </is>
       </c>
       <c r="D1827" t="inlineStr">

</xml_diff>

<commit_message>
Sync campaign design files
</commit_message>
<xml_diff>
--- a/tables/achievements.xlsx
+++ b/tables/achievements.xlsx
@@ -44753,7 +44753,7 @@
       </c>
       <c r="B862" t="inlineStr">
         <is>
-          <t>Orientation Pit: Lose initiative and still win the fight</t>
+          <t>Orientation Pit: Lost Initiative, Won Anyway</t>
         </is>
       </c>
       <c r="C862" t="inlineStr">
@@ -44793,7 +44793,7 @@
       </c>
       <c r="J862" t="inlineStr">
         <is>
-          <t>generated variant</t>
+          <t>generated variant; old name: Orientation Pit: Lose initiative and still win the fight</t>
         </is>
       </c>
     </row>
@@ -45377,7 +45377,7 @@
       </c>
       <c r="B874" t="inlineStr">
         <is>
-          <t>Orientation Pit: Destroy a camera or drone</t>
+          <t>Orientation Pit: Camera Shy</t>
         </is>
       </c>
       <c r="C874" t="inlineStr">
@@ -45417,7 +45417,7 @@
       </c>
       <c r="J874" t="inlineStr">
         <is>
-          <t>generated variant</t>
+          <t>generated variant; old name: Orientation Pit: Destroy a camera or drone</t>
         </is>
       </c>
     </row>
@@ -46521,7 +46521,7 @@
       </c>
       <c r="B896" t="inlineStr">
         <is>
-          <t>Orientation Pit: Suffer a critical failure</t>
+          <t>Orientation Pit: Critical Failure</t>
         </is>
       </c>
       <c r="C896" t="inlineStr">
@@ -46561,7 +46561,7 @@
       </c>
       <c r="J896" t="inlineStr">
         <is>
-          <t>generated variant</t>
+          <t>generated variant; old name: Orientation Pit: Suffer a critical failure</t>
         </is>
       </c>
     </row>
@@ -46677,7 +46677,7 @@
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>Orientation Pit: Refuse healing out of pride once</t>
+          <t>Orientation Pit: Too Proud to Heal</t>
         </is>
       </c>
       <c r="C899" t="inlineStr">
@@ -46717,7 +46717,7 @@
       </c>
       <c r="J899" t="inlineStr">
         <is>
-          <t>generated variant</t>
+          <t>generated variant; old name: Orientation Pit: Refuse healing out of pride once</t>
         </is>
       </c>
     </row>
@@ -46729,7 +46729,7 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>Orientation Pit: Share food with the party</t>
+          <t>Orientation Pit: Share the Snacks</t>
         </is>
       </c>
       <c r="C900" t="inlineStr">
@@ -46769,7 +46769,7 @@
       </c>
       <c r="J900" t="inlineStr">
         <is>
-          <t>generated variant</t>
+          <t>generated variant; old name: Orientation Pit: Share food with the party</t>
         </is>
       </c>
     </row>
@@ -46885,7 +46885,7 @@
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>Orientation Pit: Pay a fine</t>
+          <t>Orientation Pit: Pay a Fine</t>
         </is>
       </c>
       <c r="C903" t="inlineStr">
@@ -46925,7 +46925,7 @@
       </c>
       <c r="J903" t="inlineStr">
         <is>
-          <t>generated variant</t>
+          <t>generated variant; old name: Orientation Pit: Pay a fine</t>
         </is>
       </c>
     </row>
@@ -47041,7 +47041,7 @@
       </c>
       <c r="B906" t="inlineStr">
         <is>
-          <t>Orientation Pit: Tell the truth when a lie was safer</t>
+          <t>Orientation Pit: The Honest Option</t>
         </is>
       </c>
       <c r="C906" t="inlineStr">
@@ -47081,7 +47081,7 @@
       </c>
       <c r="J906" t="inlineStr">
         <is>
-          <t>generated variant</t>
+          <t>generated variant; old name: Orientation Pit: Tell the truth when a lie was safer</t>
         </is>
       </c>
     </row>

</xml_diff>